<commit_message>
fix: atualizar report 17-25 Set com dados corretos de respostas
Dados de resposta dos dispatches corrigidos com análise mensagem-a-mensagem
via Chatwoot API. Proposals: 3/13 responderam (23.1%). Recalls: 19/39 (48.7%).
Clínica atendeu 14 recalls e 2 proposals. 6 pacientes sem retorno da clínica.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DermaClinic_Report_17_25_Setembro.xlsx
+++ b/DermaClinic_Report_17_25_Setembro.xlsx
@@ -43,11 +43,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -65,8 +65,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -83,8 +83,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -110,12 +110,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -483,12 +483,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -528,138 +528,126 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Leads Tráfego Pago (Inbox 56)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>46</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Conversas abertas no período</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TRÁFEGO PAGO (Inbox 56)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pacientes Responderam (Inbox 56)</t>
+          <t>Leads Recebidos</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>97.8% de taxa de resposta</t>
+          <t>Conversas abertas no período</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Atendimento Humano (Inbox 56)</t>
+          <t>Pacientes Responderam</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>65.2% receberam resposta humana</t>
+          <t>97.8% taxa de resposta</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bot Only (Inbox 56)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>16</v>
+          <t>Atendimento Humano</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>30</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>34.8% ficaram apenas com bot</t>
+          <t>65.2% receberam atendente</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Agendamentos Confirmados (Inbox 56)</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
+          <t>Ficaram Apenas com Bot</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>34.8% — oportunidade perdida</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Agendamentos Confirmados</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>4.3% taxa de conversão</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Total Disparos no Período</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>321</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Todos os tipos combinados</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Disparos Birthday</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>163</v>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>100% enviados com sucesso</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>DISPAROS AUTOMÁTICOS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Disparos Confirmation</t>
+          <t>Total de Disparos</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>75</v>
+        <v>321</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>98.7% enviados</t>
+          <t>Todos os tipos no período</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Disparos Recall (Follow-up)</t>
+          <t xml:space="preserve">  Birthday</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>39</v>
+        <v>163</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -670,26 +658,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Disparos Reminder</t>
+          <t xml:space="preserve">  Confirmation</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>96.8% enviados</t>
+          <t>98.7% enviados (74/75)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Disparos Proposal</t>
+          <t xml:space="preserve">  Recall (Follow-up)</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -698,164 +686,232 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Reminder</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>31</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>96.8% enviados (30/31)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Proposals — Responderam</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>13/13</t>
-        </is>
+          <t xml:space="preserve">  Proposal (Orçamento)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>13</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100% enviados</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Proposals — Agendamentos</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>de 13 propostas</t>
-        </is>
-      </c>
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Recalls — Responderam</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>39/39</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>RESPOSTAS AOS DISPAROS</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Recalls — Agendamentos</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>7</v>
+          <t>Proposals — Responderam</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>de 39 recalls</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
+          <t>23.1% responderam</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Proposals — Clínica Atendeu</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>de 3 que responderam</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Proposals — Sem Retorno</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Paciente respondeu, clínica NÃO retornou</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>ATENDIMENTO POR RESPONSÁVEL (Inbox 56)</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Recalls — Responderam</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>19/39</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>48.7% responderam</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Responsável</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Conversas</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>% do Total</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Recalls — Clínica Atendeu</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>de 19 que responderam</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Recalls — Sem Retorno</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Paciente respondeu, clínica NÃO retornou</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ATENDIMENTO POR RESPONSÁVEL (Inbox 56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Responsável</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Conversas</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>% Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Daniela Peixer</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B31" t="n">
         <v>26</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>56.5%</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Alessandra</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B32" t="n">
         <v>13</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>28.3%</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Não atribuído</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B33" t="n">
         <v>6</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>13.0%</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Daiane Miranda da Silva</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B34" t="n">
         <v>1</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>2.2%</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -873,18 +929,18 @@
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Disparos DermaClinic — 17 a 25 de Setembro de 2026</t>
+          <t>Disparos DermaClinic — 17 a 25/Set/2026</t>
         </is>
       </c>
     </row>
@@ -922,12 +978,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Agendamentos</t>
+          <t>Clínica Atendeu</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Taxa Conversão</t>
+          <t>Sem Retorno Clínica</t>
         </is>
       </c>
     </row>
@@ -945,20 +1001,25 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -996,6 +1057,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1014,20 +1080,19 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
+      <c r="E6" t="n">
+        <v>19</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+          <t>48.7%</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>14</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -1062,6 +1127,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1080,20 +1150,19 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
+      <c r="E8" t="n">
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
+          <t>23.1%</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1113,9 +1182,20 @@
           <t>99.4%</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
+      <c r="E9" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>42.3%</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10"/>
     <row r="11"/>
@@ -1159,63 +1239,59 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Última Resposta</t>
+          <t>Resumo Resposta</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Leticia Ferreira de Lima</t>
+          <t>Patricia Ambos Pereira</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>47999374149</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>INJETAVEL VITAMINA B12</t>
-        </is>
-      </c>
+          <t>11943552185</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Oi 
+Tudo bem?
+Só gostaria de um orçamento para o laser micro agulhado
+Rosto
+Pe</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Isabel Cristina Carrara</t>
+          <t>Leticia Ferreira de Lima</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>47988991065</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>RESTYLANE + LASER CO2</t>
-        </is>
-      </c>
+          <t>47999374149</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1223,36 +1299,28 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Patricia Ambos Pereira</t>
+          <t>Isabel Cristina Carrara</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11943552185</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MEGADERME MULTILAYER + COLO + PESCOCO</t>
-        </is>
-      </c>
+          <t>47988991065</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1260,19 +1328,15 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>🤗</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1285,11 +1349,7 @@
           <t>47992250489</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>FOTONA FACE 4D</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1297,19 +1357,15 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1322,11 +1378,7 @@
           <t>47991556690</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>MMP CAPILAR + LIFTERA</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1334,19 +1386,15 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1359,31 +1407,23 @@
           <t>47999225251</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>RESTYLANE (1 SERINGA)</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>SIM</t>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1396,11 +1436,7 @@
           <t>47996046327</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>TOXINA + RESTYLANE + PEELING + SCULPTRA</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1408,19 +1444,15 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1433,11 +1465,7 @@
           <t>4899326300</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>TOXINA + RESTYLANE + SPECTRA + MEGADERME</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1445,19 +1473,15 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1470,11 +1494,7 @@
           <t>5581180622</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>CONSULTA AVALIATIVA</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -1482,19 +1502,15 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1507,11 +1523,7 @@
           <t>47999844330</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>INJETAVEL COEZIMA Q10 + B12 + MOROSIL</t>
-        </is>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -1524,12 +1536,14 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>AGENDAMENTO</t>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>pode confirmar pfvr?</t>
+          <t>boa tarde
+tudo bem e por ai?
+eu gostaria sim, veja se é possível nessa forma: qu</t>
         </is>
       </c>
     </row>
@@ -1544,11 +1558,7 @@
           <t>47988991065</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>RESTYLANE + LASER CO2</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -1556,19 +1566,15 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1581,11 +1587,7 @@
           <t>47996800800</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>FOTONA 4D</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -1593,19 +1595,15 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1618,11 +1616,7 @@
           <t>4788329691</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>MAPEAMENTO CORPORAL</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -1633,14 +1627,16 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Não anotei nada</t>
+          <t>Olá, tudo bem?
+Você pode formalizar por gentileza, a proposta
+Não anotei nada</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1682,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Última Resposta</t>
+          <t>Resumo Resposta</t>
         </is>
       </c>
     </row>
@@ -1701,11 +1697,7 @@
           <t>47999990031</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Liftera</t>
-        </is>
-      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1718,12 +1710,13 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>AGENDAMENTO</t>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>estou com uma irritação na pálpebra, tem alguma médica disponível hoje? tem aten</t>
+          <t>oi… bom dia!
+sim… quero participar da campanha.</t>
         </is>
       </c>
     </row>
@@ -1738,11 +1731,7 @@
           <t>47997297081</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Spectra</t>
-        </is>
-      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1753,14 +1742,14 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Obrigado</t>
         </is>
       </c>
     </row>
@@ -1775,11 +1764,7 @@
           <t>4789114114</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Consulta Dermatologica</t>
-        </is>
-      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>2026-09-17</t>
@@ -1787,19 +1772,15 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Obrigada pelo retorno. Assim que eu me decidir eu retorno. Tenha um ótimo dia</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1812,11 +1793,7 @@
           <t>4784206248</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Restylane</t>
-        </is>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>2026-09-19</t>
@@ -1824,19 +1801,15 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1849,11 +1822,7 @@
           <t>11972035201</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Toxina Botulinica</t>
-        </is>
-      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>2026-09-19</t>
@@ -1861,19 +1830,15 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1886,11 +1851,7 @@
           <t>554796282991</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>serviços DermaClinic</t>
-        </is>
-      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -1898,19 +1859,15 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1923,11 +1880,7 @@
           <t>554799742341</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>laser mãos</t>
-        </is>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -1935,19 +1888,15 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1960,11 +1909,7 @@
           <t>554788100789</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>consulta dermatologica</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -1972,19 +1917,15 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1997,11 +1938,7 @@
           <t>554797352457</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>avaliação dermatológica</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -2009,19 +1946,15 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2034,11 +1967,7 @@
           <t>554797349147</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>espinhas</t>
-        </is>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>2026-09-23</t>
@@ -2046,36 +1975,28 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>willian sousa</t>
+          <t>Adelir</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>554796955128</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>pele pescoço</t>
-        </is>
-      </c>
+          <t>554799728216</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2086,33 +2007,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Oi bom dia</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Raphael Galvani</t>
+          <t>Maristela</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>554797817184</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>remoção verruga</t>
-        </is>
-      </c>
+          <t>554784070004</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2120,36 +2037,28 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Marcia Rocha</t>
+          <t>willian sousa</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>554799879713</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>rejuvenescimento</t>
-        </is>
-      </c>
+          <t>554796955128</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2157,36 +2066,28 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Adelir</t>
+          <t>Raphael Galvani</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>554799728216</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>problema de pele</t>
-        </is>
-      </c>
+          <t>554797817184</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2197,33 +2098,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Gostaria de agendar consulta, convênio Unimed</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Graça</t>
+          <t>Marcia Rocha</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>554796120023</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>manchas mãos</t>
-        </is>
-      </c>
+          <t>554799879713</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2231,36 +2128,28 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Maristela</t>
+          <t>Graça</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>554784070004</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>consulta avaliativa</t>
-        </is>
-      </c>
+          <t>554796120023</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2268,36 +2157,28 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Isabela da Silveira</t>
+          <t>Marcio Marlon da Silva</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>554788729698</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>CONSULTA ISENTA</t>
-        </is>
-      </c>
+          <t>5547991784378</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2310,31 +2191,27 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>AGENDAMENTO</t>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Bom dia</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Graziela Menin</t>
+          <t>Nauan Tobias Carvalho Costa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>554799249499</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>RETORNO DR JOAO</t>
-        </is>
-      </c>
+          <t>554797197994</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2345,33 +2222,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Bom dia, obrigada</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Marlete Ribeiro</t>
+          <t>Giuliana Frohlich da Silva</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>559391016282</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Consulta + Procedimentos</t>
-        </is>
-      </c>
+          <t>5547992759212</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2382,33 +2255,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Grata!Acredito que da próxima semana ja estou melhor e entro em contato.</t>
+          <t>Boa tarde</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Marcio Marlon</t>
+          <t>Maureen Stern Weinand</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>5547991784378</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>AVALIACAO DR JOAO</t>
-        </is>
-      </c>
+          <t>554791112387</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2416,36 +2285,28 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jerry Adriano Lopes</t>
+          <t>Ledir Silvia Buchmann</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>554788606465</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>AVALIACAO DR JOAO</t>
-        </is>
-      </c>
+          <t>5547991472730</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2458,31 +2319,27 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>AGENDAMENTO</t>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Ok</t>
+          <t>Iniciei dia 28 de maio mas passei apenas 1X ao dia</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nauan Tobias</t>
+          <t>Isabela da Silveira</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>554797197994</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>FOTOTERAPIA</t>
-        </is>
-      </c>
+          <t>554788729698</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2493,33 +2350,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Conseguiu verificar com a Dra sobre um orçamento?</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Giuliana Frohlich</t>
+          <t>Graziela Menin</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>5547992759212</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>CONSULTA DERMATOLOGICA</t>
-        </is>
-      </c>
+          <t>554799249499</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2527,36 +2380,28 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Maureen Stern</t>
+          <t>Marlete Ribeiro Marques</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>554791112387</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>CONSULTA DERMATOLOGICA</t>
-        </is>
-      </c>
+          <t>559391016282</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2567,33 +2412,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Boa tarde!Cheguei esta semana,e arriei de uma bronquite passando muito ruim. Ass</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ledir Silvia Buchmann</t>
+          <t>Jerry Adriano Lopes de Oliveira</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>5547991472730</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>CONSULTA DERMATOLOGICA</t>
-        </is>
-      </c>
+          <t>554788606465</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -2604,33 +2445,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Eu vou fazer a sirujia mais vou pagar a vista eu comonico a vcs</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Esther Pilar</t>
+          <t>Leandro</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>5511945628617</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>cicatriz + clareamento</t>
-        </is>
-      </c>
+          <t>554791602825</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2641,33 +2478,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Para homens</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Sirlei De Lima</t>
+          <t>Reinert Fernanda Roberta</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>554796326338</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>limpeza Aquapur</t>
-        </is>
-      </c>
+          <t>554799955759</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2675,36 +2508,28 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Marcy Michels Ribas</t>
+          <t>Salee</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>554797625251</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>ROUCUTAN</t>
-        </is>
-      </c>
+          <t>554791248634</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2715,33 +2540,30 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t xml:space="preserve">Olá, bom dia! Tudo bem?
+Ainda estou analisando, mas assim que possível entrarei </t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Salee</t>
+          <t>Dinorah Rocha</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>554791248634</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>manchas mãos</t>
-        </is>
-      </c>
+          <t>5547999721283</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2749,36 +2571,28 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Tenha um excelente dia!</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Emanuely</t>
+          <t>Leonir Teresinha Menegheti</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>554797895565</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>marcas acne</t>
-        </is>
-      </c>
+          <t>5547992515554</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2789,33 +2603,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Pode confirmar</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dinorah Rocha</t>
+          <t>Guilherme de Araujo Ghissoni</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>5547999721283</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>MEGADERME RUGAS</t>
-        </is>
-      </c>
+          <t>5547997664848</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2823,36 +2633,28 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Leonir Teresinha</t>
+          <t>Juliana Bachmann</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>5547992515554</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>PEQUENOS PROCEDIMENTOS</t>
-        </is>
-      </c>
+          <t>5547991839222</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2863,33 +2665,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Legal já confirmo</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Guilherme Ghissoni</t>
+          <t>Liandra</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>5547997664848</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>SPECTRA TATTOO</t>
-        </is>
-      </c>
+          <t>554791928737</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2900,14 +2698,14 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Olá</t>
         </is>
       </c>
     </row>
@@ -2922,11 +2720,7 @@
           <t>554796242740</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>retirada verrugas</t>
-        </is>
-      </c>
+      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2937,33 +2731,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Muito obrigado</t>
+          <t>Olá bom dia, qual seria o valor da consulta?</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Leandro</t>
+          <t>Esther Pilar</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>554791602825</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>bioestimuladores</t>
-        </is>
-      </c>
+          <t>5511945628617</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -2971,36 +2761,28 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Reinert Fernanda</t>
+          <t>Emanuely</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>554799955759</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Consulta Dra Raquel</t>
-        </is>
-      </c>
+          <t>554797895565</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -3011,33 +2793,29 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NO_REPLY</t>
+          <t>Bom dia, tudo bem?</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Liandra</t>
+          <t>Sirlei De Lima</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>554791928737</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>flacidez XERF</t>
-        </is>
-      </c>
+          <t>554796326338</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -3045,36 +2823,28 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>AGENDAMENTO</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>tens ideia do valor?</t>
-        </is>
-      </c>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Juliana bachamn</t>
+          <t>Marcy Michels Ribas</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>5547991839222</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>consulta Dra Eoda</t>
-        </is>
-      </c>
+          <t>554797625251</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -3087,12 +2857,12 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>AGENDAMENTO</t>
+          <t>RESPONDEU - CLÍNICA ATENDEU</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Obrigada</t>
+          <t>Bom dia</t>
         </is>
       </c>
     </row>
@@ -3107,11 +2877,7 @@
           <t>554797332058</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>laser vazinhos</t>
-        </is>
-      </c>
+      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>2026-09-25</t>
@@ -3119,24 +2885,18 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>SIM</t>
+          <t>NÃO</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>RESPONDEU - SEM RETORNO DA CLÍNICA</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>NO_REPLY</t>
-        </is>
-      </c>
+          <t>SEM RESPOSTA</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A29:H29"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3155,11 +2915,11 @@
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
@@ -3242,7 +3002,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Status Conv.</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -3262,7 +3022,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Humano Atendeu?</t>
+          <t>Humano?</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -3410,7 +3170,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -3560,7 +3320,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -3710,7 +3470,7 @@
           <t>NÃO</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -3760,7 +3520,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -3956,7 +3716,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4002,7 +3762,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4048,7 +3808,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4094,7 +3854,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4240,7 +4000,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4490,7 +4250,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4740,7 +4500,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4936,7 +4696,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -4986,7 +4746,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -5086,7 +4846,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -5236,7 +4996,7 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
@@ -5554,7 +5314,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5566,21 +5326,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ações Urgentes — Oportunidades Perdidas / Follow-up Necessário</t>
+          <t>Ações Urgentes — Follow-up Necessário</t>
         </is>
       </c>
     </row>
@@ -5613,29 +5373,30 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CRÍTICA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Desiree🦋</t>
+          <t>Jessica Holz</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tráfego Pago</t>
+          <t>Proposal</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Respondeu: "Olá, tudo bem?
+Você pode formalizar por gentileza, a propost" — SEM RETORNO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Retornar URGENTE</t>
         </is>
       </c>
     </row>
@@ -5647,7 +5408,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Eva Maria</t>
+          <t>Desiree🦋</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5657,12 +5418,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5674,7 +5435,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sofia Prevedello</t>
+          <t>Eva Maria</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5684,12 +5445,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5462,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>🩺Fonoaudióloga Lívia🧩🎧🦻</t>
+          <t>Sofia Prevedello</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5711,12 +5472,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5728,7 +5489,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cristina</t>
+          <t>🩺Fonoaudióloga Lívia🧩🎧🦻</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5738,12 +5499,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5755,7 +5516,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Claudio Krieck</t>
+          <t>Cristina</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5765,12 +5526,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5543,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Schirlei Vieira Gonçalves</t>
+          <t>Claudio Krieck</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5792,12 +5553,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5809,7 +5570,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Terezinha</t>
+          <t>Schirlei Vieira Gonçalves</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5819,12 +5580,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5597,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Giselle Camilo</t>
+          <t>Terezinha</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5846,12 +5607,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5624,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>😂</t>
+          <t>Giselle Camilo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -5873,12 +5634,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5651,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ana Cristina</t>
+          <t>😂</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5900,12 +5661,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5917,7 +5678,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gabriela Maria Branco</t>
+          <t>Ana Cristina</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5927,12 +5688,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5705,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Michella Marinho</t>
+          <t>Gabriela Maria Branco</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5954,12 +5715,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5732,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Claudia Ribas (🌻)</t>
+          <t>Michella Marinho</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5981,12 +5742,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -5998,7 +5759,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Salee</t>
+          <t>Claudia Ribas (🌻)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -6008,12 +5769,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -6025,7 +5786,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Esther Pilar</t>
+          <t>Salee</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -6035,12 +5796,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Lead respondeu mas ficou só com bot</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Atribuir a atendente e retornar contato</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
@@ -6052,61 +5813,61 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Leticia Ferreira de Lima</t>
+          <t>Esther Pilar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Proposal</t>
+          <t>Tráfego Pago</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Respondeu ao follow-up de INJETAVEL VITAMINA B12 mas não agendou</t>
+          <t>Lead respondeu mas ficou apenas com bot</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Contato pessoal para fechar agendamento</t>
+          <t>Atribuir atendente e retornar</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Patricia Dias Birckholz</t>
+          <t>EDNA CARGNIM ROGÉRIO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Proposal</t>
+          <t>Recall</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Respondeu ao follow-up de RESTYLANE (1 SERINGA) mas não agendou</t>
+          <t>Respondeu ao recall de  — sem retorno</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Contato pessoal para fechar agendamento</t>
+          <t>Verificar conversa e retornar</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>MÉDIA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EDNA CARGNIM ROGÉRIO</t>
+          <t>Adelir</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -6116,7 +5877,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Respondeu ao recall de Spectra sem retorno da clínica</t>
+          <t>Respondeu ao recall de  — sem retorno</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -6126,14 +5887,14 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>MÉDIA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Elaine</t>
+          <t>Leandro</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6143,7 +5904,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Respondeu ao recall de Consulta Dermatologica sem retorno da clínica</t>
+          <t>Respondeu ao recall de  — sem retorno</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -6153,14 +5914,14 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>MÉDIA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Hye Jin Kim</t>
+          <t>Salee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -6170,7 +5931,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Respondeu ao recall de Toxina Botulinica sem retorno da clínica</t>
+          <t>Respondeu ao recall de  — sem retorno</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6180,14 +5941,14 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>MÉDIA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Sofia Prevedello</t>
+          <t>Emanuely</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -6197,172 +5958,10 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Respondeu ao recall de serviços DermaClinic sem retorno da clínica</t>
+          <t>Respondeu ao recall de  — sem retorno</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
-        <is>
-          <t>Verificar conversa e retornar</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Vivi</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Respondeu ao recall de laser mãos sem retorno da clínica</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Verificar conversa e retornar</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Suely Maria</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Respondeu ao recall de consulta dermatologica sem retorno da clínica</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Verificar conversa e retornar</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Brenda</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Respondeu ao recall de avaliação dermatológica sem retorno da clínica</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Verificar conversa e retornar</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Kamila</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Respondeu ao recall de espinhas sem retorno da clínica</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Verificar conversa e retornar</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>willian sousa</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Respondeu ao recall de pele pescoço sem retorno da clínica</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Verificar conversa e retornar</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Raphael Galvani</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Respondeu ao recall de remoção verruga sem retorno da clínica</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
         <is>
           <t>Verificar conversa e retornar</t>
         </is>
@@ -6385,14 +5984,14 @@
   <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
@@ -6400,7 +5999,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Inbox 56 — Conversas Setembro 17-25</t>
+          <t>Inbox 56 — Conversas 17-25 Set</t>
         </is>
       </c>
     </row>
@@ -6438,12 +6037,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Msgs Incoming</t>
+          <t>Incoming</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Msgs Outgoing</t>
+          <t>Outgoing</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -8566,7 +8165,7 @@
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -8579,7 +8178,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Disparos por Dia — 17 a 25 de Setembro de 2026</t>
+          <t>Disparos por Dia — 17 a 25/Set/2026</t>
         </is>
       </c>
     </row>
@@ -8624,7 +8223,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>17/09</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -8649,7 +8248,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>18/09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -8674,7 +8273,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>19/09</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -8699,7 +8298,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>20/09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -8724,7 +8323,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>21/09</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -8749,7 +8348,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>22/09</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -8774,7 +8373,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>23/09</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -8799,7 +8398,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>24/09</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -8824,7 +8423,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>25/09</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -8917,36 +8516,36 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Fonte — Tráfego Pago</t>
+          <t>Fonte Tráfego Pago</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chatwoot API — Inbox 56 (Tráfego Pago), Account 4</t>
+          <t>Chatwoot API — Inbox 56, Account 4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Fonte — Disparos</t>
+          <t>Fonte Disparos</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PostgreSQL dermaclinic — tabela recall_tasks (dispatched_at no período)</t>
+          <t>PostgreSQL dermaclinic — recall_tasks (dispatched_at)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Fonte — Respostas</t>
+          <t>Fonte Respostas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chatwoot API — conversas por contato, msgs após data de disparo</t>
+          <t>Chatwoot API — conversas do contato, mensagens pós-disparo</t>
         </is>
       </c>
     </row>
@@ -8958,7 +8557,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>patient_responded = msg_type 0 presente; human_responded = msg_type 1 com sender User; bot_only = sem humano; agendou = label contém 'agend'</t>
+          <t>patient_responded = msg incoming; human_responded = msg outgoing de User; agendou = label 'agend'</t>
         </is>
       </c>
     </row>
@@ -8970,7 +8569,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>responded = msg_type 0 (incoming) após cutoff; clinic_responded = msg_type 1 (User) após incoming; AGENDAMENTO = label com 'agend'</t>
+          <t>responded = msg incoming após data disparo; clinic_responded = msg outgoing de User após resposta</t>
         </is>
       </c>
     </row>
@@ -8982,7 +8581,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Respostas via ligação telefônica não captadas. Agendamentos sem label no Chatwoot podem não ser contados. Conversas de proposals sem contact_id foram buscadas por telefone.</t>
+          <t>Respostas por telefone/presencial não captadas. Agendamentos sem label podem não ser contados.</t>
         </is>
       </c>
     </row>
@@ -8994,19 +8593,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DAI — Digital AI (automação)</t>
+          <t>DAI — Digital AI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Data de geração</t>
+          <t>Data geração</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-25 16:31</t>
+          <t>2026-09-25 16:34</t>
         </is>
       </c>
     </row>

</xml_diff>